<commit_message>
feat(templates,abap): support Profit Center ALPHA conversion, Person Responsible padding, and PS_ACTVT expansion
</commit_message>
<xml_diff>
--- a/excel-templates/Template_Role.xlsx
+++ b/excel-templates/Template_Role.xlsx
@@ -808,24 +808,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -853,7 +855,7 @@
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>Profit Center</t>
+          <t>Profit Center (C_PROJ_PRC, C_PRPS_PRC)</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
@@ -889,6 +891,16 @@
       <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Costing variant (K_KEKO)</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Person Responsible (C_PROJ_VNR-PS_VERNR, C_PRPS_VNR-PS_VERNR)</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>Project System (Field PS_ACTVT)</t>
         </is>
       </c>
     </row>
@@ -930,14 +942,14 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>10000100 - 10009899; ' '</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>1000*</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>1000*</t>
-        </is>
-      </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>*</t>
@@ -964,6 +976,16 @@
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>00000000; 00000080</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>*</t>
         </is>
@@ -1007,14 +1029,14 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
+          <t>' '</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
           <t>2000*</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>2000*</t>
-        </is>
-      </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>*</t>
@@ -1043,6 +1065,16 @@
       <c r="O3" s="3" t="inlineStr">
         <is>
           <t>*</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>03, F4</t>
         </is>
       </c>
     </row>
@@ -1084,14 +1116,14 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>10009930; ' '</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>1000*</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>1000*</t>
-        </is>
-      </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>*</t>
@@ -1122,98 +1154,56 @@
           <t>*</t>
         </is>
       </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>00000000;</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Z_FI_GL_MASTER_MAINT</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Z_FI_GL_MASTER_MAINT_2000</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>GL Master Data Maint - CC 2000</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>2000*</t>
-        </is>
-      </c>
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2000*</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
+      <c r="P5" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Z_FI_JOURNAL_POST</t>
+          <t>Z_FI_GL_MASTER_MAINT</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Z_FI_JOURNAL_POST_1000</t>
+          <t>Z_FI_GL_MASTER_MAINT_2000</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>General Ledger Posting - CC 1000</t>
+          <t>GL Master Data Maint - CC 2000</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1228,22 +1218,22 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>1000*</t>
+          <t>20000100 - 20009899; ' '</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>1000*</t>
+          <t>2000*</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -1274,6 +1264,16 @@
       <c r="O6" s="3" t="inlineStr">
         <is>
           <t>*</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>03, F4</t>
         </is>
       </c>
     </row>
@@ -1285,70 +1285,167 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>Z_FI_JOURNAL_POST_1000</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>General Ledger Posting - CC 1000</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>1000*</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>1000*</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Z_FI_JOURNAL_POST</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>Z_FI_JOURNAL_POST_2000</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>General Ledger Posting - CC 2000</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>2000*</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>2000*</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>*</t>
         </is>

</xml_diff>

<commit_message>
feat(scripts): support Col 4 activity conversion and include master roles in object levels
</commit_message>
<xml_diff>
--- a/excel-templates/Template_Role.xlsx
+++ b/excel-templates/Template_Role.xlsx
@@ -833,74 +833,74 @@
     <row r="1">
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>ACTVT, PS_ACTVT</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
           <t>Operating concern
 ($CEERKRS)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Controlling area
 ($KOKRS)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Company Code ($BUKRS)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Plant / Valuation Area</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Profit Center (C_PROJ_PRC, C_PRPS_PRC)</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Cost center</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Order type</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Asset Class</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Business Place</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Credit segment</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>Costing variant (K_KEKO)</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>Person Responsible (C_PROJ_VNR-PS_VERNR, C_PRPS_VNR-PS_VERNR)</t>
-        </is>
-      </c>
-      <c r="Q1" s="4" t="inlineStr">
-        <is>
-          <t>Project System (Field PS_ACTVT)</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>*</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -942,19 +942,19 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>10000100 - 10009899; ' '</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>1000*</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>*</t>
@@ -982,12 +982,12 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
           <t>00000000; 00000080</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>03, F4</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1019,29 +1019,29 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>' '</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>2000*</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>*</t>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>03, F4</t>
+          <t>*</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>*</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1116,19 +1116,19 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>10009930; ' '</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>1000*</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>*</t>
@@ -1156,12 +1156,12 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
           <t>00000000;</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
         </is>
       </c>
     </row>
@@ -1174,21 +1174,21 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
-      <c r="P5" s="3" t="n">
+      <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="Q5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>03, F4</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1218,29 +1218,29 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>20000100 - 20009899; ' '</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>2000*</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
           <t>*</t>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>03, F4</t>
+          <t>*</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>*</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1315,17 +1315,17 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
           <t>1000*</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>1000*</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>*</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1392,27 +1392,27 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>2000*</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>2000*</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>*</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">

</xml_diff>